<commit_message>
Gemma's DeepInfra repair finishes clean: 112 unusable rows -> 0
All 20 tasks now on disk, the 5 repaired ones on DeepInfra with seed=42 and the
other 15 untouched on Together. Every one of the 112 rows that were empty or
missing the Final Answer marker on Together came back usable: causal_judgement
3->0, date_understanding 4->0, dyck_languages 41->0, formal_fallacies 22->0,
geometric_shapes 42->0. formal_fallacies alone moved 0.912 -> 1.000.

Macro-average 0.9493 -> 0.9684. Final_Result.xlsx updated.

Qwen's 13-task repair is still running in the background.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Final_Result.xlsx
+++ b/Final_Result.xlsx
@@ -591,7 +591,7 @@
         <v>0.615</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.6898</v>
+        <v>0.6952</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0.6791</v>
@@ -616,7 +616,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0.9399999999999999</v>
@@ -641,7 +641,7 @@
         <v>0.516</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.828</v>
+        <v>0.956</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0.856</v>
@@ -666,7 +666,7 @@
         <v>0.968</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.912</v>
+        <v>1</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1</v>
@@ -691,7 +691,7 @@
         <v>0.8</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.648</v>
+        <v>0.804</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0.8</v>
@@ -1066,7 +1066,7 @@
         <v>0.9101</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0.9493</v>
+        <v>0.9684</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>0.9616</v>

</xml_diff>